<commit_message>
Canvi en "desglosDeParticions" no repartia correctament les particions orig en els traspassos.
</commit_message>
<xml_diff>
--- a/Docs/ProvesMetode-CompresDeParticions2.xlsx
+++ b/Docs/ProvesMetode-CompresDeParticions2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63189381-B823-422F-8298-77A3C5E61BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE137AF-4C60-4698-8BA2-25FBCBEDD5D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{9C88047F-F2B0-4C94-90F2-1B9BFBAFCCBB}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="76">
   <si>
     <t>Data Compra Orig</t>
   </si>
@@ -205,6 +205,66 @@
   </si>
   <si>
     <t>xx</t>
+  </si>
+  <si>
+    <t>Acció</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Tarsp A-C</t>
+  </si>
+  <si>
+    <t>Tarsp B-C</t>
+  </si>
+  <si>
+    <t>Acc Orig</t>
+  </si>
+  <si>
+    <t>Venda C</t>
+  </si>
+  <si>
+    <t>Venudes</t>
+  </si>
+  <si>
+    <t>Queden</t>
+  </si>
+  <si>
+    <t>Mov</t>
+  </si>
+  <si>
+    <t>MovOrig</t>
+  </si>
+  <si>
+    <t>Parts desg</t>
+  </si>
+  <si>
+    <t>Parts Orig desg</t>
+  </si>
+  <si>
+    <t>En les vendes seran les particions del mov sense desgloçar</t>
+  </si>
+  <si>
+    <t>Data Orig</t>
+  </si>
+  <si>
+    <t>En les vendes será la del Mov.</t>
+  </si>
+  <si>
+    <t>Parts Ocupades</t>
+  </si>
+  <si>
+    <t>Parts disponibles</t>
+  </si>
+  <si>
+    <t>Parts Utilitzades</t>
+  </si>
+  <si>
+    <t>Parts Utili Orig</t>
+  </si>
+  <si>
+    <t>Struct</t>
   </si>
 </sst>
 </file>
@@ -241,7 +301,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +329,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -322,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -399,6 +471,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -713,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E44D0EF9-1D37-4AF3-8267-1950FB3DB311}">
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.90625" bestFit="1" customWidth="1"/>
@@ -724,9 +798,12 @@
     <col min="6" max="6" width="10.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="10.6328125" customWidth="1"/>
     <col min="9" max="9" width="1.7265625" customWidth="1"/>
+    <col min="10" max="10" width="14.81640625" customWidth="1"/>
+    <col min="12" max="12" width="10.36328125" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>4</v>
       </c>
@@ -745,8 +822,23 @@
       </c>
       <c r="G1" s="11"/>
       <c r="H1" s="11"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="M1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>26</v>
       </c>
@@ -771,8 +863,26 @@
         <f>D2</f>
         <v>249.34710000000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" s="48">
+        <v>1</v>
+      </c>
+      <c r="P2" s="48">
+        <v>10</v>
+      </c>
+      <c r="Q2" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>28</v>
       </c>
@@ -797,33 +907,91 @@
         <f>IF(ISNUMBER(SEARCH("v",B3,1)),J2-D3,J2+D3)</f>
         <v>0.34710000000001173</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="O3" s="48">
+        <v>2</v>
+      </c>
+      <c r="P3" s="48">
+        <v>100</v>
+      </c>
+      <c r="Q3" s="48">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C4" s="2"/>
       <c r="D4" s="25"/>
       <c r="E4" s="20"/>
       <c r="F4" s="20"/>
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L4" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O4">
+        <v>3</v>
+      </c>
+      <c r="Q4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C5" s="2"/>
       <c r="D5" s="25"/>
       <c r="E5" s="20"/>
       <c r="F5" s="20"/>
       <c r="G5" s="20"/>
       <c r="H5" s="20"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="N5" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="O5" s="48">
+        <v>2</v>
+      </c>
+      <c r="P5" s="48">
+        <v>50</v>
+      </c>
+      <c r="Q5" s="48">
+        <f>Q4</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C6" s="2"/>
       <c r="D6" s="25"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L7" t="s">
+        <v>58</v>
+      </c>
+      <c r="M7" t="s">
+        <v>39</v>
+      </c>
+      <c r="O7">
+        <v>4</v>
+      </c>
+      <c r="Q7">
+        <v>400</v>
+      </c>
+      <c r="R7">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>15</v>
       </c>
@@ -836,8 +1004,19 @@
       <c r="E8">
         <v>39.353999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="N8" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8" s="48"/>
+      <c r="P8" s="48">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="48">
+        <f>Q7</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>15</v>
       </c>
@@ -850,8 +1029,21 @@
       <c r="E9">
         <v>679.64</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="N9" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="O9" s="48">
+        <v>2</v>
+      </c>
+      <c r="P9" s="48">
+        <v>50</v>
+      </c>
+      <c r="Q9" s="48">
+        <f>Q5</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>15</v>
       </c>
@@ -865,7 +1057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>15</v>
       </c>
@@ -878,8 +1070,33 @@
       <c r="E11">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L11" t="s">
+        <v>61</v>
+      </c>
+      <c r="M11" t="s">
+        <v>39</v>
+      </c>
+      <c r="O11">
+        <v>5</v>
+      </c>
+      <c r="Q11">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="N12" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12" s="49"/>
+      <c r="P12" s="49">
+        <f>Q12/Q8*P8</f>
+        <v>3.75</v>
+      </c>
+      <c r="Q12" s="49">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>16</v>
       </c>
@@ -892,8 +1109,20 @@
       <c r="E13">
         <v>76.952299999999994</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="N13" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13" s="48"/>
+      <c r="P13" s="48">
+        <f>P8-P12</f>
+        <v>6.25</v>
+      </c>
+      <c r="Q13" s="48">
+        <f>Q8-Q12</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>16</v>
       </c>
@@ -906,8 +1135,22 @@
       <c r="E14">
         <v>547.64509999999996</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="N14" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="O14" s="48">
+        <v>2</v>
+      </c>
+      <c r="P14" s="48">
+        <f>P9</f>
+        <v>50</v>
+      </c>
+      <c r="Q14" s="48">
+        <f>Q9</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>16</v>
       </c>
@@ -921,7 +1164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>16</v>
       </c>
@@ -935,7 +1178,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="L17" t="s">
+        <v>61</v>
+      </c>
+      <c r="M17" t="s">
+        <v>39</v>
+      </c>
+      <c r="O17">
+        <v>6</v>
+      </c>
+      <c r="Q17">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>17</v>
       </c>
@@ -954,8 +1211,20 @@
       <c r="H18">
         <v>141.64619999999999</v>
       </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="N18" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18" s="49"/>
+      <c r="P18" s="49">
+        <f>P12</f>
+        <v>3.75</v>
+      </c>
+      <c r="Q18" s="49">
+        <f>Q12</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>17</v>
       </c>
@@ -974,8 +1243,20 @@
       <c r="H19">
         <v>1008.0512</v>
       </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="N19" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="O19" s="49"/>
+      <c r="P19" s="49">
+        <f>Q19/Q14*P14</f>
+        <v>25</v>
+      </c>
+      <c r="Q19" s="49">
+        <f>Q17-Q18</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B20">
         <v>17</v>
       </c>
@@ -994,8 +1275,19 @@
       <c r="H20">
         <v>141.64619999999999</v>
       </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="N20" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20" s="48"/>
+      <c r="P20" s="48">
+        <f>Q20/Q12*P12</f>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B21">
         <v>17</v>
       </c>
@@ -1014,8 +1306,30 @@
       <c r="H21">
         <v>1008.0512</v>
       </c>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="L21" s="49" t="s">
+        <v>62</v>
+      </c>
+      <c r="N21" s="48" t="s">
+        <v>57</v>
+      </c>
+      <c r="O21" s="48">
+        <v>2</v>
+      </c>
+      <c r="P21" s="48">
+        <f>P14-P19</f>
+        <v>25</v>
+      </c>
+      <c r="Q21" s="48">
+        <f>Q14-Q19</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="L22" s="48" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B23">
         <v>15</v>
       </c>
@@ -1023,7 +1337,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>15</v>
       </c>
@@ -1031,7 +1345,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B25">
         <v>15</v>
       </c>
@@ -1039,71 +1353,111 @@
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B26">
         <v>15</v>
       </c>
       <c r="C26" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="J26" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="J27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B28">
         <v>16</v>
       </c>
       <c r="C28" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="J28" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>16</v>
       </c>
       <c r="C29" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="J29" t="s">
+        <v>69</v>
+      </c>
+      <c r="K29" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B30">
         <v>16</v>
       </c>
       <c r="C30" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="J30" t="s">
+        <v>66</v>
+      </c>
+      <c r="K30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B31">
         <v>16</v>
       </c>
       <c r="C31" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="J31" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="J32" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B33">
         <v>17</v>
       </c>
       <c r="C33" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="J33" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B34">
         <v>17</v>
       </c>
       <c r="C34" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="J34" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B35">
         <v>17</v>
       </c>
       <c r="C35" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="J35" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B36">
         <v>17</v>
       </c>
@@ -1111,7 +1465,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B38">
         <v>27</v>
       </c>
@@ -1125,7 +1479,7 @@
         <v>6.2279999999999998</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B39">
         <v>27</v>
       </c>
@@ -1139,7 +1493,7 @@
         <v>56.674100000000003</v>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B40">
         <v>27</v>
       </c>
@@ -1153,7 +1507,7 @@
         <v>1.23029999999997</v>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B41">
         <v>27</v>
       </c>
@@ -1167,12 +1521,12 @@
         <v>11.195591719652899</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B44">
         <v>17</v>
       </c>
@@ -1183,7 +1537,7 @@
         <v>137.07740000000001</v>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B45">
         <v>17</v>
       </c>
@@ -1194,7 +1548,7 @@
         <v>1010.611</v>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B46">
         <v>17</v>
       </c>
@@ -1205,7 +1559,7 @@
         <v>116.65349999999999</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B47">
         <v>17</v>
       </c>
@@ -3093,7 +3447,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCF58976-EAE7-4A0A-A776-E4303DC2CBF0}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.54296875" style="1" customWidth="1"/>
@@ -3548,6 +3902,158 @@
         <v>4.997600000000034</v>
       </c>
       <c r="M19" s="19"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="D21" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B22" s="8">
+        <v>92</v>
+      </c>
+      <c r="C22">
+        <v>15</v>
+      </c>
+      <c r="D22">
+        <v>443.13400000000001</v>
+      </c>
+      <c r="E22">
+        <v>679.64009999999996</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B23" s="8">
+        <v>92</v>
+      </c>
+      <c r="C23">
+        <v>16</v>
+      </c>
+      <c r="D23">
+        <v>866.49839999999995</v>
+      </c>
+      <c r="E23">
+        <v>547.64509999999996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B24" s="8">
+        <v>92</v>
+      </c>
+      <c r="C24">
+        <v>17</v>
+      </c>
+      <c r="D24">
+        <v>1596.6121000000001</v>
+      </c>
+      <c r="E24">
+        <v>1009.1815</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B25" s="8">
+        <v>92</v>
+      </c>
+      <c r="C25">
+        <v>27</v>
+      </c>
+      <c r="D25">
+        <v>16.115600000000001</v>
+      </c>
+      <c r="E25">
+        <v>13.0237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B27">
+        <v>92</v>
+      </c>
+      <c r="C27">
+        <v>15</v>
+      </c>
+      <c r="D27">
+        <v>443.13400000000001</v>
+      </c>
+      <c r="E27">
+        <v>679.64</v>
+      </c>
+      <c r="F27">
+        <f>+D27-D22</f>
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <f>+E27-E22</f>
+        <v>-9.9999999974897946E-5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B28">
+        <v>92</v>
+      </c>
+      <c r="C28">
+        <v>16</v>
+      </c>
+      <c r="D28">
+        <v>866.49839999999995</v>
+      </c>
+      <c r="E28">
+        <v>547.64509999999996</v>
+      </c>
+      <c r="F28">
+        <f t="shared" ref="F28:G28" si="2">+D28-D23</f>
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B29">
+        <v>92</v>
+      </c>
+      <c r="C29">
+        <v>17</v>
+      </c>
+      <c r="D29">
+        <v>1598.8742</v>
+      </c>
+      <c r="E29">
+        <v>1010.611</v>
+      </c>
+      <c r="F29">
+        <f t="shared" ref="F29:G29" si="3">+D29-D24</f>
+        <v>2.2620999999999185</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="3"/>
+        <v>1.4294999999999618</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B30">
+        <v>92</v>
+      </c>
+      <c r="C30">
+        <v>27</v>
+      </c>
+      <c r="D30">
+        <v>13.853400000000001</v>
+      </c>
+      <c r="E30">
+        <v>11.195600000000001</v>
+      </c>
+      <c r="F30">
+        <f t="shared" ref="F30:G30" si="4">+D30-D25</f>
+        <v>-2.2622</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="4"/>
+        <v>-1.8280999999999992</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>